<commit_message>
Fix BUG-001 (destructive import) and BUG-004 (fail-open authorization)
BUG-001 — CustomerSegmentation.runImport no longer deletes the entire
customer_yearly_sales table before inserting. It now upserts on
(customer_code, year, region_name) in batches and asks for confirmation
first, so a mid-run failure can never lose data and re-running is
idempotent.

BUG-004 — App.js now fails closed on authorization. getNav() returns an
empty nav (not NAV_ADMIN) for an unknown/missing role, and renderPage()
gates the admin page switch behind role === 'admin', showing a new
NoAccess screen for any unknown/null role instead of exposing admin pages.

Updated qa-reports bug report/change log to mark both as fixed. Verified:
79/79 unit tests pass, ESLint clean (no new warnings), build compiles.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UKgs9YA8dwySKm4rWeUEMm
</commit_message>
<xml_diff>
--- a/qa-reports/06-bug-report.xlsx
+++ b/qa-reports/06-bug-report.xlsx
@@ -419,7 +419,7 @@
     <col min="13" max="13" width="60.83203125" customWidth="1"/>
     <col min="14" max="14" width="60.83203125" customWidth="1"/>
     <col min="15" max="15" width="22.83203125" customWidth="1"/>
-    <col min="16" max="16" width="40.83203125" customWidth="1"/>
+    <col min="16" max="16" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,7 +519,7 @@
         <v>TC-055</v>
       </c>
       <c r="P2" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — import now upsert-only + confirm</v>
       </c>
     </row>
     <row r="3">
@@ -669,7 +669,7 @@
         <v>TC-010</v>
       </c>
       <c r="P5" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — fail-closed role, NoAccess screen</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Update QA bug statuses and change log after the full fix run
Mark 30 bugs Fixed, 2 Partially fixed (BUG-005 parser hardening pending a
dependency upgrade; BUG-029 test infra + first test), and 2 Deferred
needing input (BUG-020 server-side aggregation, BUG-022 grading decision).
Regenerate 06-bug-report.xlsx and record the full Sprint 1-3 change log.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UKgs9YA8dwySKm4rWeUEMm
</commit_message>
<xml_diff>
--- a/qa-reports/06-bug-report.xlsx
+++ b/qa-reports/06-bug-report.xlsx
@@ -519,7 +519,7 @@
         <v>TC-055</v>
       </c>
       <c r="P2" t="str">
-        <v>Fixed (branch claude/dashboard-review-5oyboy) — import now upsert-only + confirm</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — import upsert-only + confirm</v>
       </c>
     </row>
     <row r="3">
@@ -569,7 +569,7 @@
         <v>TC-030</v>
       </c>
       <c r="P3" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — deactivate-before-split + full compensation</v>
       </c>
     </row>
     <row r="4">
@@ -619,7 +619,7 @@
         <v>TC-020</v>
       </c>
       <c r="P4" t="str">
-        <v>Open (needs DB verification)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — year/month written explicitly (DB verify still advised)</v>
       </c>
     </row>
     <row r="5">
@@ -669,7 +669,7 @@
         <v>TC-010</v>
       </c>
       <c r="P5" t="str">
-        <v>Fixed (branch claude/dashboard-review-5oyboy) — fail-closed role, NoAccess screen</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — fail-closed role + NoAccess screen</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +719,7 @@
         <v>TC-063</v>
       </c>
       <c r="P6" t="str">
-        <v>Open (confirmed by npm audit)</v>
+        <v>Partially fixed — parser hardened (type/size/row caps, try-catch); dependency upgrade still required at deploy</v>
       </c>
     </row>
     <row r="7">
@@ -769,7 +769,7 @@
         <v>TC-045</v>
       </c>
       <c r="P7" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — totals relabeled to all-time</v>
       </c>
     </row>
     <row r="8">
@@ -819,7 +819,7 @@
         <v>TC-050</v>
       </c>
       <c r="P8" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — dynamic-year chart/headers + div-by-zero guard</v>
       </c>
     </row>
     <row r="9">
@@ -869,7 +869,7 @@
         <v>TC-051</v>
       </c>
       <c r="P9" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — null-name guard + ComposedChart</v>
       </c>
     </row>
     <row r="10">
@@ -919,7 +919,7 @@
         <v>TC-041</v>
       </c>
       <c r="P10" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — KPI uses selected-month progress</v>
       </c>
     </row>
     <row r="11">
@@ -969,7 +969,7 @@
         <v>TC-042</v>
       </c>
       <c r="P11" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — shelf_photos aggregated + correct column</v>
       </c>
     </row>
     <row r="12">
@@ -1019,7 +1019,7 @@
         <v>TC-043</v>
       </c>
       <c r="P12" t="str">
-        <v>Open (partially fixed in RepDashboard)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — month-phase daily-required in Dashboard &amp; RepDetails</v>
       </c>
     </row>
     <row r="13">
@@ -1069,7 +1069,7 @@
         <v>TC-021</v>
       </c>
       <c r="P13" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — daily-entry &amp; targets validation</v>
       </c>
     </row>
     <row r="14">
@@ -1119,7 +1119,7 @@
         <v>TC-022</v>
       </c>
       <c r="P14" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — month/year selectors read-only</v>
       </c>
     </row>
     <row r="15">
@@ -1169,7 +1169,7 @@
         <v>TC-023</v>
       </c>
       <c r="P15" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — local-date default</v>
       </c>
     </row>
     <row r="16">
@@ -1219,7 +1219,7 @@
         <v>TC-031</v>
       </c>
       <c r="P16" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — Setup mutations check errors</v>
       </c>
     </row>
     <row r="17">
@@ -1269,7 +1269,7 @@
         <v>TC-032</v>
       </c>
       <c r="P17" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — crypto temp password</v>
       </c>
     </row>
     <row r="18">
@@ -1319,7 +1319,7 @@
         <v>TC-035</v>
       </c>
       <c r="P18" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — audit error capture + page_view throttle</v>
       </c>
     </row>
     <row r="19">
@@ -1369,7 +1369,7 @@
         <v>TC-036</v>
       </c>
       <c r="P19" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — today-stats from dedicated query</v>
       </c>
     </row>
     <row r="20">
@@ -1419,7 +1419,7 @@
         <v>TC-025</v>
       </c>
       <c r="P20" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — Targets fetch scoped to on-or-before month</v>
       </c>
     </row>
     <row r="21">
@@ -1469,7 +1469,7 @@
         <v>TC-060</v>
       </c>
       <c r="P21" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Open (deferred) — needs server-side aggregation/pagination (Customers/Segmentation still client-side; Targets over-fetch fixed)</v>
       </c>
     </row>
     <row r="22">
@@ -1519,7 +1519,7 @@
         <v>TC-052</v>
       </c>
       <c r="P22" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — ABC/Pareto clear data + error state</v>
       </c>
     </row>
     <row r="23">
@@ -1569,7 +1569,7 @@
         <v>TC-053</v>
       </c>
       <c r="P23" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Open (deferred) — needs product decision on one canonical grading definition</v>
       </c>
     </row>
     <row r="24">
@@ -1619,7 +1619,7 @@
         <v>TC-026</v>
       </c>
       <c r="P24" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — create/update keyed off real month target</v>
       </c>
     </row>
     <row r="25">
@@ -1669,7 +1669,7 @@
         <v>TC-033</v>
       </c>
       <c r="P25" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — inherited target not split on handover</v>
       </c>
     </row>
     <row r="26">
@@ -1719,7 +1719,7 @@
         <v>TC-046</v>
       </c>
       <c r="P26" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — Customers scoping fails closed</v>
       </c>
     </row>
     <row r="27">
@@ -1769,7 +1769,7 @@
         <v>TC-070</v>
       </c>
       <c r="P27" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — error states + import parse handling</v>
       </c>
     </row>
     <row r="28">
@@ -1819,7 +1819,7 @@
         <v>TC-024</v>
       </c>
       <c r="P28" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — daily-entry overwrite confirm</v>
       </c>
     </row>
     <row r="29">
@@ -1869,7 +1869,7 @@
         <v>TC-065</v>
       </c>
       <c r="P29" t="str">
-        <v>Open (confirmed by lint)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — 0 ESLint warnings; CI build gate passes</v>
       </c>
     </row>
     <row r="30">
@@ -1919,7 +1919,7 @@
         <v>TC-066</v>
       </c>
       <c r="P30" t="str">
-        <v>Open (confirmed by coverage)</v>
+        <v>Partially fixed — component-test infra + first ChangePassword test (more component/E2E tests pending)</v>
       </c>
     </row>
     <row r="31">
@@ -1969,7 +1969,7 @@
         <v>TC-044</v>
       </c>
       <c r="P31" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — fetch cancellation guards</v>
       </c>
     </row>
     <row r="32">
@@ -2019,7 +2019,7 @@
         <v>TC-064</v>
       </c>
       <c r="P32" t="str">
-        <v>Open (confirmed)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — build/ removed from VCS + gitignored</v>
       </c>
     </row>
     <row r="33">
@@ -2069,7 +2069,7 @@
         <v>TC-037</v>
       </c>
       <c r="P33" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — Gregorian calendar</v>
       </c>
     </row>
     <row r="34">
@@ -2119,7 +2119,7 @@
         <v>TC-054</v>
       </c>
       <c r="P34" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — data-aligned years; compare previous year</v>
       </c>
     </row>
     <row r="35">
@@ -2169,7 +2169,7 @@
         <v>TC-005</v>
       </c>
       <c r="P35" t="str">
-        <v>Open (confirmed by static review)</v>
+        <v>Fixed (branch claude/dashboard-review-5oyboy) — email format + stronger password policy</v>
       </c>
     </row>
   </sheetData>

</xml_diff>